<commit_message>
style(templates): add title row to Excel templates
- Add merged title row to clock_table, reset_table, sub_clock_table
- Title format: '时钟树/复位树/子时钟树配置表 (xxx Configuration)'
- Restore wechat_article.md from backup
</commit_message>
<xml_diff>
--- a/cr_tree_diag_gen/examples/input/clock_table.xlsx
+++ b/cr_tree_diag_gen/examples/input/clock_table.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -193,8 +193,14 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill/>
     </fill>
@@ -391,6 +397,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5496"/>
+        <bgColor rgb="002F5496"/>
       </patternFill>
     </fill>
   </fills>
@@ -663,7 +675,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -673,6 +685,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1086,7 +1101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1104,94 +1119,79 @@
     <col width="11" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>时钟树配置表 (Clock Tree Configuration)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>NAME</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>SEL</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>SRC0</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>SRC1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>MUX_DFLT</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>DIV</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>DIV_WIDTH</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>DIV_DFLT</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>OCC</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>ICG</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K2" s="1" t="inlineStr">
         <is>
           <t>ICG_DFLT</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L2" s="1" t="inlineStr">
         <is>
           <t>ATTR</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>test_mode</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>input</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>pll_src_clk</t>
+          <t>test_mode</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr"/>
@@ -1213,7 +1213,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>apb_src_clk</t>
+          <t>pll_src_clk</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr"/>
@@ -1235,7 +1235,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>pad_src_clk</t>
+          <t>apb_src_clk</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr"/>
@@ -1257,7 +1257,7 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>div_src_clk</t>
+          <t>pad_src_clk</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr"/>
@@ -1279,7 +1279,7 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Clock Generate</t>
+          <t>div_src_clk</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr"/>
@@ -1292,46 +1292,34 @@
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>core_clk</t>
+          <t>Clock Generate</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>apb_src_clk</t>
-        </is>
-      </c>
+      <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L8" s="3" t="inlineStr">
-        <is>
-          <t>output</t>
-        </is>
-      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>peri_clk</t>
+          <t>core_clk</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr"/>
@@ -1365,7 +1353,7 @@
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>dbg_pclk</t>
+          <t>peri_clk</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr"/>
@@ -1399,7 +1387,7 @@
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>cfg_clk</t>
+          <t>dbg_pclk</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr"/>
@@ -1414,8 +1402,16 @@
       <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr"/>
       <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
           <t>output</t>
@@ -1425,7 +1421,7 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>io_pclk</t>
+          <t>cfg_clk</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr"/>
@@ -1440,16 +1436,8 @@
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="3" t="inlineStr">
         <is>
           <t>output</t>
@@ -1459,33 +1447,21 @@
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>vol_clk</t>
+          <t>io_pclk</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr"/>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>pad_src_clk</t>
+          <t>apb_src_clk</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>clk_divider</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>OCC</t>
-        </is>
-      </c>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1505,21 +1481,33 @@
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>vol_pclk</t>
+          <t>vol_clk</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>apb_src_clk</t>
+          <t>pad_src_clk</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>clk_divider</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1539,7 +1527,7 @@
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>mon_clk</t>
+          <t>vol_pclk</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr"/>
@@ -1573,13 +1561,13 @@
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>efuse_ref</t>
+          <t>mon_clk</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr"/>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>pad_src_clk</t>
+          <t>apb_src_clk</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
@@ -1607,13 +1595,13 @@
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>efuse_pclk</t>
+          <t>efuse_ref</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr"/>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>apb_src_clk</t>
+          <t>pad_src_clk</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
@@ -1641,13 +1629,13 @@
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>sub_ref</t>
+          <t>efuse_pclk</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr"/>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>pad_src_clk</t>
+          <t>apb_src_clk</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
@@ -1661,17 +1649,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>internal</t>
+          <t>output</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>s32k_clk</t>
+          <t>sub_ref</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr"/>
@@ -1682,34 +1674,26 @@
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>clk_divider</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>OCC</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>output</t>
+          <t>internal</t>
         </is>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ref_clk</t>
+          <t>s32k_clk</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr"/>
@@ -1720,10 +1704,22 @@
       </c>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>clk_divider</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="3" t="inlineStr">
@@ -1735,7 +1731,7 @@
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>sec_ref</t>
+          <t>ref_clk</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr"/>
@@ -1754,60 +1750,40 @@
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>internal</t>
+          <t>output</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>trace_clk</t>
+          <t>sec_ref</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr"/>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>pll_src_clk</t>
+          <t>pad_src_clk</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>clk_divider</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H22" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>OCC</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>output</t>
+          <t>internal</t>
         </is>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>sys_pll</t>
+          <t>trace_clk</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr"/>
@@ -1818,10 +1794,22 @@
       </c>
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr"/>
-      <c r="H23" s="2" t="inlineStr"/>
-      <c r="I23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>clk_divider</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1841,13 +1829,13 @@
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>top_ref</t>
+          <t>sys_pll</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>pad_src_clk</t>
+          <t>pll_src_clk</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
@@ -1875,33 +1863,21 @@
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>rom_div</t>
+          <t>top_ref</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr"/>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>div_src_clk</t>
+          <t>pad_src_clk</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>clk_divider_er</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H25" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>OCC</t>
-        </is>
-      </c>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1921,27 +1897,43 @@
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>gpio_det</t>
+          <t>rom_div</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr"/>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>pad_src_clk</t>
+          <t>div_src_clk</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>clk_divider_er</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
           <t>output</t>
@@ -1951,43 +1943,27 @@
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>trng_clk</t>
+          <t>gpio_det</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr"/>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>pll_src_clk</t>
+          <t>pad_src_clk</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>clk_divider</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H27" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>OCC</t>
-        </is>
-      </c>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="3" t="inlineStr">
         <is>
           <t>output</t>
@@ -1997,7 +1973,7 @@
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>pll_test</t>
+          <t>trng_clk</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr"/>
@@ -2017,30 +1993,79 @@
         <v>8</v>
       </c>
       <c r="H28" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>pll_test</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>pll_src_clk</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>clk_divider</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H29" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>OCC</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L28" s="3" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L29" s="3" t="inlineStr">
         <is>
           <t>output</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>